<commit_message>
Sem: 24.04.2026 ödemesini Nisan ayına taşı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USLtU2rCVCG4DPBtXYDA9a
</commit_message>
<xml_diff>
--- a/borc_takip_2026.xlsx
+++ b/borc_takip_2026.xlsx
@@ -982,27 +982,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>25.05.2026</t>
+          <t>24.04.2026</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>60000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>60000</v>
-      </c>
-      <c r="E5" s="3">
+        <v>20000</v>
+      </c>
+      <c r="E5" s="4">
         <f>C5-D5</f>
         <v/>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Hesaptan</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Borç yok</t>
+          <t>~445$; 40.000 kalan (defterde yer olmadığı için en alta yazılmış)</t>
         </is>
       </c>
     </row>
@@ -1014,16 +1014,16 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>28.06.2026</t>
+          <t>25.05.2026</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>60000</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E6" s="4">
+        <v>60000</v>
+      </c>
+      <c r="E6" s="3">
         <f>C6-D6</f>
         <v/>
       </c>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>10.000 kalan</t>
+          <t>Borç yok</t>
         </is>
       </c>
     </row>
@@ -1046,14 +1046,14 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>24.07.2026</t>
+          <t>28.06.2026</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
         <v>60000</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="E7" s="4">
         <f>C7-D7</f>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>20.000 kalan</t>
+          <t>10.000 kalan</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>29.08.2026</t>
+          <t>24.07.2026</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
@@ -1110,14 +1110,14 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>23.09.2026</t>
+          <t>29.08.2026</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>60000</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="E9" s="4">
         <f>C9-D9</f>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>10.000 kalan</t>
+          <t>20.000 kalan</t>
         </is>
       </c>
     </row>
@@ -1142,14 +1142,14 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>24.04.2026 (?)</t>
+          <t>23.09.2026</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>60000</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E10" s="4">
         <f>C10-D10</f>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>Hesaptan</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>~445$; defterde tarih 24.04 yazıyor, sıraya göre 24.09/24.10 olmalı — kontrol edin</t>
+          <t>10.000 kalan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel dosyasını Google Sheets sürümüyle eşitle
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USLtU2rCVCG4DPBtXYDA9a
</commit_message>
<xml_diff>
--- a/borc_takip_2026.xlsx
+++ b/borc_takip_2026.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0&quot; TL&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +30,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -65,38 +70,45 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00BFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00BFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00BFBFBF"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFD8A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -461,13 +473,13 @@
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -608,7 +620,7 @@
       <c r="D5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <f>C5-D5</f>
         <v/>
       </c>
@@ -632,7 +644,7 @@
       <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <f>C6-D6</f>
         <v/>
       </c>
@@ -656,7 +668,7 @@
       <c r="D7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <f>C7-D7</f>
         <v/>
       </c>
@@ -684,7 +696,7 @@
       <c r="D8" s="3" t="n">
         <v>40000</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <f>C8-D8</f>
         <v/>
       </c>
@@ -716,7 +728,7 @@
       <c r="D9" s="3" t="n">
         <v>40000</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <f>C9-D9</f>
         <v/>
       </c>
@@ -748,7 +760,7 @@
       <c r="D10" s="3" t="n">
         <v>40000</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <f>C10-D10</f>
         <v/>
       </c>
@@ -776,7 +788,7 @@
       <c r="D11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <f>C11-D11</f>
         <v/>
       </c>
@@ -797,28 +809,33 @@
       <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOPLAM</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="6">
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="5">
         <f>SUM(C2:C11)</f>
         <v/>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <f>SUM(D2:D11)</f>
         <v/>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <f>SUM(E2:E11)</f>
         <v/>
       </c>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E11">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -832,13 +849,13 @@
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -924,8 +941,9 @@
       <c r="C3" s="3" t="n">
         <v>60000</v>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>60000</v>
+      <c r="D3" s="3">
+        <f>26500+33500</f>
+        <v/>
       </c>
       <c r="E3" s="3">
         <f>C3-D3</f>
@@ -938,7 +956,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>600$ = 26.500 + 750$ = 33.500 — borç yok</t>
+          <t>600$ = 26.500 TL ve 750$ = 33.500 TL, borç yok</t>
         </is>
       </c>
     </row>
@@ -991,7 +1009,7 @@
       <c r="D5" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <f>C5-D5</f>
         <v/>
       </c>
@@ -1002,7 +1020,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>~445$; 40.000 kalan (defterde yer olmadığı için en alta yazılmış)</t>
+          <t>Yaklaşık 445$, 40.000 kalan (defterde en alta yazılmış)</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1073,7 @@
       <c r="D7" s="3" t="n">
         <v>50000</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <f>C7-D7</f>
         <v/>
       </c>
@@ -1087,7 +1105,7 @@
       <c r="D8" s="3" t="n">
         <v>40000</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <f>C8-D8</f>
         <v/>
       </c>
@@ -1119,7 +1137,7 @@
       <c r="D9" s="3" t="n">
         <v>40000</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <f>C9-D9</f>
         <v/>
       </c>
@@ -1151,7 +1169,7 @@
       <c r="D10" s="3" t="n">
         <v>50000</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <f>C10-D10</f>
         <v/>
       </c>
@@ -1179,7 +1197,7 @@
       <c r="D11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <f>C11-D11</f>
         <v/>
       </c>
@@ -1200,28 +1218,33 @@
       <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOPLAM</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="6">
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="5">
         <f>SUM(C2:C11)</f>
         <v/>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <f>SUM(D2:D11)</f>
         <v/>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <f>SUM(E2:E11)</f>
         <v/>
       </c>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E11">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1232,57 +1255,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Kişi</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Toplam Borç (26.10.2026)</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Toplam Ödenen (TL)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Toplam Borç (TL)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Tarih</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Cem</t>
         </is>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="3">
+        <f>Cem!D13</f>
+        <v/>
+      </c>
+      <c r="C2" s="3">
         <f>Cem!E13</f>
         <v/>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Sem</t>
         </is>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="3">
+        <f>Sem!D13</f>
+        <v/>
+      </c>
+      <c r="C3" s="3">
         <f>Sem!E13</f>
         <v/>
       </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="5">
         <f>B2+B3</f>
         <v/>
       </c>
+      <c r="C4" s="6">
+        <f>C2+C3</f>
+        <v/>
+      </c>
+      <c r="D4" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>